<commit_message>
Working on understanding Henrique's needs
</commit_message>
<xml_diff>
--- a/report_scripts/Matos Henrique/Other kerosene and Fuel oil example.xlsx
+++ b/report_scripts/Matos Henrique/Other kerosene and Fuel oil example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/PFUPipeline2/report_scripts/Matos Henrique/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D908212-21C2-B245-A44B-FC7E5D44DFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C00836-EB0E-F14D-9419-BCCA53DEF3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2460" yWindow="860" windowWidth="40320" windowHeight="33900" activeTab="1" xr2:uid="{C9C58493-B417-3A4E-803E-79C3192C4023}"/>
+    <workbookView xWindow="-29400" yWindow="9780" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{C9C58493-B417-3A4E-803E-79C3192C4023}"/>
   </bookViews>
   <sheets>
     <sheet name="Other kerosene" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="96">
   <si>
     <t>Other kerosene -&gt; Residential</t>
   </si>
@@ -376,12 +376,6 @@
     <t>Fuel oil -&gt; Industry not elsewhere specified</t>
   </si>
   <si>
-    <t xml:space="preserve">Y_final |&gt; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  matsbyname::fractionize_byname(Y_final, margin = 2) |&gt; </t>
-  </si>
-  <si>
     <t xml:space="preserve">  matsbyname::vectorize_byname(notation = RCLabels::arrow_notation) |&gt;</t>
   </si>
   <si>
@@ -407,13 +401,22 @@
   </si>
   <si>
     <t>Y_f_special</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  matsbyname::fractionize_byname(margin = 2) |&gt; </t>
+  </si>
+  <si>
+    <t>Convert column notation from "from notation" to "arrow notation"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y_f |&gt; </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -426,6 +429,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -456,8 +466,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFD3712D"/>
       </patternFill>
     </fill>
   </fills>
@@ -470,10 +479,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
@@ -497,10 +507,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -510,9 +516,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{21FD03A4-B495-EA4A-9752-52290E2FE97C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1710,6 +1720,118 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>105</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>1143000</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Straight Arrow Connector 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5158D514-677C-2D4C-B20B-94BC253E9C18}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34226500" y="5194300"/>
+          <a:ext cx="57759600" cy="7670800"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="50800">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>99</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>102</xdr:col>
+      <xdr:colOff>711200</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="10" name="Straight Arrow Connector 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65AB1C9D-04F6-334F-86EB-9A9ABF224F11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="87045800" y="15494000"/>
+          <a:ext cx="2997200" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="50800">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2126,10 +2248,10 @@
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="12"/>
+      <c r="C9" s="10"/>
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2164,14 +2286,14 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="12"/>
-      <c r="N10" s="12" t="s">
+      <c r="H10" s="10"/>
+      <c r="N10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="O10" s="12"/>
+      <c r="O10" s="10"/>
       <c r="Z10" s="8" t="s">
         <v>25</v>
       </c>
@@ -2355,25 +2477,25 @@
       <c r="C19" s="7">
         <v>0</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
-      <c r="N19" s="12" t="s">
+      <c r="N19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-      <c r="Q19" s="12"/>
-      <c r="U19" s="12" t="s">
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="U19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="V19" s="12"/>
-      <c r="W19" s="12"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
       <c r="X19" s="8"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
@@ -2386,21 +2508,21 @@
       <c r="C20" s="7">
         <v>175.20079999999999</v>
       </c>
-      <c r="N20" s="13" t="s">
+      <c r="N20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="O20" s="13"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="11"/>
       <c r="U20" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="12"/>
+      <c r="C21" s="10"/>
     </row>
     <row r="31" spans="1:24" ht="129" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
@@ -2535,11 +2657,11 @@
       <c r="B36" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G36" s="12" t="s">
+      <c r="G36" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
       <c r="M36" s="2" t="s">
         <v>1</v>
       </c>
@@ -2555,11 +2677,11 @@
       <c r="Q36" s="4"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="N37" s="12" t="s">
+      <c r="N37" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="O37" s="12"/>
-      <c r="P37" s="12"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
       <c r="Q37" s="8"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
@@ -2587,7 +2709,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89C181D5-361B-AB4A-B6A7-B6C14CEC1F09}">
-  <dimension ref="A2:DR93"/>
+  <dimension ref="A2:DT93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" bestFit="1" customWidth="1"/>
@@ -2655,22 +2777,22 @@
       <c r="A3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="12">
         <v>80.399100000000004</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="12">
         <v>7437</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="12">
         <v>924.60040000000004</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="12">
         <v>3698.4009999999998</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="12">
         <v>200.9999</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="12">
         <v>321.60070000000002</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -2719,14 +2841,14 @@
       </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
       <c r="J4" s="2" t="s">
         <v>34</v>
       </c>
@@ -2957,22 +3079,22 @@
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="K9" s="12" t="s">
+      <c r="K9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="AH9" s="12" t="s">
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="AH9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="AI9" s="12"/>
-      <c r="AJ9" s="12"/>
-      <c r="AK9" s="12"/>
-      <c r="AL9" s="12"/>
-      <c r="AM9" s="12"/>
+      <c r="AI9" s="10"/>
+      <c r="AJ9" s="10"/>
+      <c r="AK9" s="10"/>
+      <c r="AL9" s="10"/>
+      <c r="AM9" s="10"/>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.2">
       <c r="K10" s="5"/>
@@ -3195,7 +3317,7 @@
       <c r="AL16" s="5"/>
       <c r="AM16" s="5"/>
     </row>
-    <row r="17" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>38</v>
       </c>
@@ -3230,16 +3352,16 @@
       <c r="AL17" s="5"/>
       <c r="AM17" s="5"/>
     </row>
-    <row r="18" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="B18" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
@@ -3253,10 +3375,10 @@
       <c r="AL18" s="5"/>
       <c r="AM18" s="5"/>
     </row>
-    <row r="19" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="11" t="s">
-        <v>84</v>
+      <c r="B19" s="9" t="s">
+        <v>95</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3276,10 +3398,10 @@
       <c r="AL19" s="5"/>
       <c r="AM19" s="5"/>
     </row>
-    <row r="20" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="11" t="s">
-        <v>85</v>
+      <c r="B20" s="9" t="s">
+        <v>93</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3299,10 +3421,10 @@
       <c r="AL20" s="5"/>
       <c r="AM20" s="5"/>
     </row>
-    <row r="21" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="11" t="s">
-        <v>86</v>
+      <c r="B21" s="9" t="s">
+        <v>84</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -3322,10 +3444,10 @@
       <c r="AL21" s="5"/>
       <c r="AM21" s="5"/>
     </row>
-    <row r="22" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="11" t="s">
-        <v>87</v>
+      <c r="B22" s="9" t="s">
+        <v>85</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -3345,9 +3467,9 @@
       <c r="AL22" s="5"/>
       <c r="AM22" s="5"/>
     </row>
-    <row r="23" spans="1:122" x14ac:dyDescent="0.2">
-      <c r="B23" s="11" t="s">
-        <v>88</v>
+    <row r="23" spans="1:124" x14ac:dyDescent="0.2">
+      <c r="B23" s="9" t="s">
+        <v>86</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
@@ -3362,9 +3484,9 @@
       <c r="AL23" s="5"/>
       <c r="AM23" s="5"/>
     </row>
-    <row r="24" spans="1:122" x14ac:dyDescent="0.2">
-      <c r="B24" s="11" t="s">
-        <v>89</v>
+    <row r="24" spans="1:124" x14ac:dyDescent="0.2">
+      <c r="B24" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
@@ -3379,9 +3501,9 @@
       <c r="AL24" s="5"/>
       <c r="AM24" s="5"/>
     </row>
-    <row r="25" spans="1:122" x14ac:dyDescent="0.2">
-      <c r="B25" s="11" t="s">
-        <v>90</v>
+    <row r="25" spans="1:124" x14ac:dyDescent="0.2">
+      <c r="B25" s="9" t="s">
+        <v>88</v>
       </c>
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
@@ -3396,7 +3518,7 @@
       <c r="AL25" s="5"/>
       <c r="AM25" s="5"/>
     </row>
-    <row r="30" spans="1:122" ht="263" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:124" ht="263" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
         <v>28</v>
       </c>
@@ -3707,26 +3829,26 @@
         <v>78</v>
       </c>
     </row>
-    <row r="31" spans="1:122" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:124" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="6">
-        <v>0</v>
-      </c>
-      <c r="C31" s="6">
+      <c r="B31" s="12">
+        <v>0</v>
+      </c>
+      <c r="C31" s="12">
         <v>7437.0002999999997</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="12">
         <v>924.60040000000004</v>
       </c>
-      <c r="E31" s="6">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6">
-        <v>0</v>
-      </c>
-      <c r="G31" s="6">
+      <c r="E31" s="12">
+        <v>0</v>
+      </c>
+      <c r="F31" s="12">
+        <v>0</v>
+      </c>
+      <c r="G31" s="12">
         <v>321.60070000000002</v>
       </c>
       <c r="J31" s="2" t="s">
@@ -4059,27 +4181,31 @@
       <c r="DR31" s="6">
         <v>0</v>
       </c>
+      <c r="DT31">
+        <f t="shared" ref="DT31:DT33" si="1">SUM(CZ31:DR31)</f>
+        <v>0.99999998619378805</v>
+      </c>
     </row>
-    <row r="32" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B32" s="6">
-        <v>0</v>
-      </c>
-      <c r="C32" s="6">
-        <v>0</v>
-      </c>
-      <c r="D32" s="6">
-        <v>0</v>
-      </c>
-      <c r="E32" s="6">
+      <c r="B32" s="12">
+        <v>0</v>
+      </c>
+      <c r="C32" s="12">
+        <v>0</v>
+      </c>
+      <c r="D32" s="12">
+        <v>0</v>
+      </c>
+      <c r="E32" s="12">
         <v>45.420974487803001</v>
       </c>
-      <c r="F32" s="6">
-        <v>0</v>
-      </c>
-      <c r="G32" s="6">
+      <c r="F32" s="12">
+        <v>0</v>
+      </c>
+      <c r="G32" s="12">
         <v>0</v>
       </c>
       <c r="J32" s="2" t="s">
@@ -4149,83 +4275,83 @@
         <v>29</v>
       </c>
       <c r="AH32" s="6">
-        <f t="shared" ref="AH32:AH36" si="1">K32</f>
+        <f t="shared" ref="AH32:AH36" si="2">K32</f>
         <v>7437.0002999999997</v>
       </c>
       <c r="AI32" s="6">
-        <f t="shared" ref="AI32:AI36" si="2">L32</f>
+        <f t="shared" ref="AI32:AI36" si="3">L32</f>
         <v>0</v>
       </c>
       <c r="AJ32" s="6">
-        <f t="shared" ref="AJ32:AJ36" si="3">M32</f>
+        <f t="shared" ref="AJ32:AJ36" si="4">M32</f>
         <v>0</v>
       </c>
       <c r="AK32" s="6">
-        <f t="shared" ref="AK32:AK36" si="4">N32</f>
+        <f t="shared" ref="AK32:AK36" si="5">N32</f>
         <v>0</v>
       </c>
       <c r="AL32" s="6">
-        <f t="shared" ref="AL32:AL36" si="5">O32</f>
+        <f t="shared" ref="AL32:AL36" si="6">O32</f>
         <v>0</v>
       </c>
       <c r="AM32" s="6">
-        <f t="shared" ref="AM32:AM36" si="6">P32</f>
+        <f t="shared" ref="AM32:AM36" si="7">P32</f>
         <v>0</v>
       </c>
       <c r="AN32" s="6">
-        <f t="shared" ref="AN32:AN36" si="7">Q32</f>
+        <f t="shared" ref="AN32:AN36" si="8">Q32</f>
         <v>0</v>
       </c>
       <c r="AO32" s="6">
-        <f t="shared" ref="AO32:AO36" si="8">R32</f>
+        <f t="shared" ref="AO32:AO36" si="9">R32</f>
         <v>0</v>
       </c>
       <c r="AP32" s="6">
-        <f t="shared" ref="AP32:AP36" si="9">S32</f>
+        <f t="shared" ref="AP32:AP36" si="10">S32</f>
         <v>0</v>
       </c>
       <c r="AQ32" s="6">
-        <f t="shared" ref="AQ32:AQ36" si="10">T32</f>
+        <f t="shared" ref="AQ32:AQ36" si="11">T32</f>
         <v>0</v>
       </c>
       <c r="AR32" s="6">
-        <f t="shared" ref="AR32:AR36" si="11">U32</f>
+        <f t="shared" ref="AR32:AR36" si="12">U32</f>
         <v>0</v>
       </c>
       <c r="AS32" s="6">
-        <f t="shared" ref="AS32:AS36" si="12">V32</f>
+        <f t="shared" ref="AS32:AS36" si="13">V32</f>
         <v>0</v>
       </c>
       <c r="AT32" s="6">
-        <f t="shared" ref="AT32:AT36" si="13">W32</f>
+        <f t="shared" ref="AT32:AT36" si="14">W32</f>
         <v>0</v>
       </c>
       <c r="AU32" s="6">
-        <f t="shared" ref="AU32:AU36" si="14">X32</f>
+        <f t="shared" ref="AU32:AU36" si="15">X32</f>
         <v>0</v>
       </c>
       <c r="AV32" s="6">
-        <f t="shared" ref="AV32:AV36" si="15">Y32</f>
+        <f t="shared" ref="AV32:AV36" si="16">Y32</f>
         <v>0</v>
       </c>
       <c r="AW32" s="6">
-        <f t="shared" ref="AW32:AW36" si="16">Z32</f>
+        <f t="shared" ref="AW32:AW36" si="17">Z32</f>
         <v>0</v>
       </c>
       <c r="AX32" s="6">
-        <f t="shared" ref="AX32:AX36" si="17">AA32</f>
+        <f t="shared" ref="AX32:AX36" si="18">AA32</f>
         <v>0</v>
       </c>
       <c r="AY32" s="6">
-        <f t="shared" ref="AY32:AY36" si="18">AB32</f>
+        <f t="shared" ref="AY32:AY36" si="19">AB32</f>
         <v>0</v>
       </c>
       <c r="AZ32" s="6">
-        <f t="shared" ref="AZ32:AZ36" si="19">AC32</f>
+        <f t="shared" ref="AZ32:AZ36" si="20">AC32</f>
         <v>0</v>
       </c>
       <c r="BA32" s="6">
-        <f t="shared" ref="BA32:BA36" si="20">AD32</f>
+        <f t="shared" ref="BA32:BA36" si="21">AD32</f>
         <v>0</v>
       </c>
       <c r="BD32" s="2" t="s">
@@ -4408,27 +4534,31 @@
       <c r="DR32" s="6">
         <v>0</v>
       </c>
+      <c r="DT32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B33" s="6">
-        <v>0</v>
-      </c>
-      <c r="C33" s="6">
-        <v>0</v>
-      </c>
-      <c r="D33" s="6">
-        <v>0</v>
-      </c>
-      <c r="E33" s="6">
+      <c r="B33" s="12">
+        <v>0</v>
+      </c>
+      <c r="C33" s="12">
+        <v>0</v>
+      </c>
+      <c r="D33" s="12">
+        <v>0</v>
+      </c>
+      <c r="E33" s="12">
         <v>10.56548974729</v>
       </c>
-      <c r="F33" s="6">
-        <v>0</v>
-      </c>
-      <c r="G33" s="6">
+      <c r="F33" s="12">
+        <v>0</v>
+      </c>
+      <c r="G33" s="12">
         <v>0</v>
       </c>
       <c r="J33" s="2" t="s">
@@ -4498,83 +4628,83 @@
         <v>30</v>
       </c>
       <c r="AH33" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>924.60040000000004</v>
       </c>
       <c r="AI33" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AJ33" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AK33" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AL33" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AM33" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AN33" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AO33" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AP33" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AQ33" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AR33" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AS33" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AT33" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AU33" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AV33" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AW33" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX33" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="AY33" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="AZ33" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="BA33" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="BD33" s="2" t="s">
@@ -4757,27 +4887,31 @@
       <c r="DR33" s="6">
         <v>0</v>
       </c>
+      <c r="DT33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B34" s="6">
-        <v>0</v>
-      </c>
-      <c r="C34" s="6">
-        <v>0</v>
-      </c>
-      <c r="D34" s="6">
-        <v>0</v>
-      </c>
-      <c r="E34" s="6">
+      <c r="B34" s="12">
+        <v>0</v>
+      </c>
+      <c r="C34" s="12">
+        <v>0</v>
+      </c>
+      <c r="D34" s="12">
+        <v>0</v>
+      </c>
+      <c r="E34" s="12">
         <v>239.42002754622999</v>
       </c>
-      <c r="F34" s="6">
-        <v>0</v>
-      </c>
-      <c r="G34" s="6">
+      <c r="F34" s="12">
+        <v>0</v>
+      </c>
+      <c r="G34" s="12">
         <v>0</v>
       </c>
       <c r="J34" s="2" t="s">
@@ -4847,83 +4981,83 @@
         <v>39</v>
       </c>
       <c r="AH34" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI34" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>45.420974487803001</v>
       </c>
       <c r="AJ34" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.56548974729</v>
       </c>
       <c r="AK34" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>239.42002754622999</v>
       </c>
       <c r="AL34" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>320.41223929520999</v>
       </c>
       <c r="AM34" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>13.894729834892001</v>
       </c>
       <c r="AN34" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>134.58699587643</v>
       </c>
       <c r="AO34" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>4.8328734732758001</v>
       </c>
       <c r="AP34" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>2.4537243968652998E-2</v>
       </c>
       <c r="AQ34" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>66.682419111564002</v>
       </c>
       <c r="AR34" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>20.72619293088</v>
       </c>
       <c r="AS34" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>11.722790773811001</v>
       </c>
       <c r="AT34" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>351.12025842441</v>
       </c>
       <c r="AU34" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>10.981003594759001</v>
       </c>
       <c r="AV34" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>4.7239291045123002</v>
       </c>
       <c r="AW34" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX34" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1855.3143386280001</v>
       </c>
       <c r="AY34" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>73.809561478158003</v>
       </c>
       <c r="AZ34" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="BA34" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>2.1592437759009999</v>
       </c>
       <c r="BD34" s="2" t="s">
@@ -5106,27 +5240,31 @@
       <c r="DR34" s="6">
         <v>2.9659791716219358E-4</v>
       </c>
+      <c r="DT34">
+        <f>SUM(CZ34:DR34)</f>
+        <v>1.0000001066217485</v>
+      </c>
     </row>
-    <row r="35" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B35" s="6">
-        <v>0</v>
-      </c>
-      <c r="C35" s="6">
-        <v>0</v>
-      </c>
-      <c r="D35" s="6">
-        <v>0</v>
-      </c>
-      <c r="E35" s="6">
+      <c r="B35" s="12">
+        <v>0</v>
+      </c>
+      <c r="C35" s="12">
+        <v>0</v>
+      </c>
+      <c r="D35" s="12">
+        <v>0</v>
+      </c>
+      <c r="E35" s="12">
         <v>320.41223929520999</v>
       </c>
-      <c r="F35" s="6">
-        <v>0</v>
-      </c>
-      <c r="G35" s="6">
+      <c r="F35" s="12">
+        <v>0</v>
+      </c>
+      <c r="G35" s="12">
         <v>0</v>
       </c>
       <c r="J35" s="2" t="s">
@@ -5196,83 +5334,83 @@
         <v>31</v>
       </c>
       <c r="AH35" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI35" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AJ35" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AK35" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AL35" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AM35" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AN35" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AO35" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AP35" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AQ35" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AR35" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AS35" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AT35" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AU35" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AV35" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AW35" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX35" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="AY35" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="AZ35" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>171.94047456000001</v>
       </c>
       <c r="BA35" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="BD35" s="2" t="s">
@@ -5455,27 +5593,31 @@
       <c r="DR35" s="6">
         <v>0</v>
       </c>
+      <c r="DT35">
+        <f t="shared" ref="DT35:DT36" si="22">SUM(CZ35:DR35)</f>
+        <v>1.0000000000000004</v>
+      </c>
     </row>
-    <row r="36" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B36" s="6">
-        <v>0</v>
-      </c>
-      <c r="C36" s="6">
-        <v>0</v>
-      </c>
-      <c r="D36" s="6">
-        <v>0</v>
-      </c>
-      <c r="E36" s="6">
+      <c r="B36" s="12">
+        <v>0</v>
+      </c>
+      <c r="C36" s="12">
+        <v>0</v>
+      </c>
+      <c r="D36" s="12">
+        <v>0</v>
+      </c>
+      <c r="E36" s="12">
         <v>13.894729834892001</v>
       </c>
-      <c r="F36" s="6">
-        <v>0</v>
-      </c>
-      <c r="G36" s="6">
+      <c r="F36" s="12">
+        <v>0</v>
+      </c>
+      <c r="G36" s="12">
         <v>0</v>
       </c>
       <c r="J36" s="2" t="s">
@@ -5545,83 +5687,83 @@
         <v>32</v>
       </c>
       <c r="AH36" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>321.60070000000002</v>
       </c>
       <c r="AI36" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AJ36" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AK36" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AL36" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AM36" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AN36" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AO36" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AP36" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AQ36" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AR36" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AS36" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AT36" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AU36" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AV36" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AW36" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX36" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="AY36" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="AZ36" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="BA36" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="BD36" s="2" t="s">
@@ -5804,414 +5946,421 @@
       <c r="DR36" s="6">
         <v>0</v>
       </c>
+      <c r="DT36">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="6">
-        <v>0</v>
-      </c>
-      <c r="C37" s="6">
-        <v>0</v>
-      </c>
-      <c r="D37" s="6">
-        <v>0</v>
-      </c>
-      <c r="E37" s="6">
+      <c r="B37" s="12">
+        <v>0</v>
+      </c>
+      <c r="C37" s="12">
+        <v>0</v>
+      </c>
+      <c r="D37" s="12">
+        <v>0</v>
+      </c>
+      <c r="E37" s="12">
         <v>134.58699587643</v>
       </c>
-      <c r="F37" s="6">
-        <v>0</v>
-      </c>
-      <c r="G37" s="6">
-        <v>0</v>
-      </c>
-      <c r="K37" s="12" t="s">
+      <c r="F37" s="12">
+        <v>0</v>
+      </c>
+      <c r="G37" s="12">
+        <v>0</v>
+      </c>
+      <c r="K37" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="L37" s="12"/>
-      <c r="M37" s="12"/>
-      <c r="N37" s="12"/>
-      <c r="O37" s="12"/>
-      <c r="P37" s="12"/>
-      <c r="Q37" s="12"/>
-      <c r="R37" s="12"/>
-      <c r="S37" s="12"/>
-      <c r="T37" s="12"/>
-      <c r="U37" s="12"/>
-      <c r="V37" s="12"/>
-      <c r="W37" s="12"/>
-      <c r="X37" s="12"/>
-      <c r="Y37" s="12"/>
-      <c r="Z37" s="12"/>
-      <c r="AA37" s="12"/>
-      <c r="AB37" s="12"/>
-      <c r="AC37" s="12"/>
-      <c r="AD37" s="12"/>
-      <c r="AH37" s="12" t="s">
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="10"/>
+      <c r="S37" s="10"/>
+      <c r="T37" s="10"/>
+      <c r="U37" s="10"/>
+      <c r="V37" s="10"/>
+      <c r="W37" s="10"/>
+      <c r="X37" s="10"/>
+      <c r="Y37" s="10"/>
+      <c r="Z37" s="10"/>
+      <c r="AA37" s="10"/>
+      <c r="AB37" s="10"/>
+      <c r="AC37" s="10"/>
+      <c r="AD37" s="10"/>
+      <c r="AH37" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="AI37" s="12"/>
-      <c r="AJ37" s="12"/>
-      <c r="AK37" s="12"/>
-      <c r="AL37" s="12"/>
-      <c r="AM37" s="12"/>
-      <c r="AN37" s="12"/>
-      <c r="AO37" s="12"/>
-      <c r="AP37" s="12"/>
-      <c r="AQ37" s="12"/>
-      <c r="AR37" s="12"/>
-      <c r="AS37" s="12"/>
-      <c r="AT37" s="12"/>
-      <c r="AU37" s="12"/>
-      <c r="AV37" s="12"/>
-      <c r="AW37" s="12"/>
-      <c r="AX37" s="12"/>
-      <c r="AY37" s="12"/>
-      <c r="AZ37" s="12"/>
-      <c r="BA37" s="12"/>
-      <c r="BE37" s="12" t="s">
+      <c r="AI37" s="10"/>
+      <c r="AJ37" s="10"/>
+      <c r="AK37" s="10"/>
+      <c r="AL37" s="10"/>
+      <c r="AM37" s="10"/>
+      <c r="AN37" s="10"/>
+      <c r="AO37" s="10"/>
+      <c r="AP37" s="10"/>
+      <c r="AQ37" s="10"/>
+      <c r="AR37" s="10"/>
+      <c r="AS37" s="10"/>
+      <c r="AT37" s="10"/>
+      <c r="AU37" s="10"/>
+      <c r="AV37" s="10"/>
+      <c r="AW37" s="10"/>
+      <c r="AX37" s="10"/>
+      <c r="AY37" s="10"/>
+      <c r="AZ37" s="10"/>
+      <c r="BA37" s="10"/>
+      <c r="BE37" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="BF37" s="12"/>
-      <c r="BG37" s="12"/>
-      <c r="BH37" s="12"/>
-      <c r="BI37" s="12"/>
-      <c r="BJ37" s="12"/>
-      <c r="BK37" s="12"/>
-      <c r="BL37" s="12"/>
-      <c r="BM37" s="12"/>
-      <c r="BN37" s="12"/>
-      <c r="BO37" s="12"/>
-      <c r="BP37" s="12"/>
-      <c r="BQ37" s="12"/>
-      <c r="BR37" s="12"/>
-      <c r="BS37" s="12"/>
-      <c r="BT37" s="12"/>
-      <c r="BU37" s="12"/>
-      <c r="BV37" s="12"/>
-      <c r="BW37" s="12"/>
-      <c r="CC37" s="12" t="s">
+      <c r="BF37" s="10"/>
+      <c r="BG37" s="10"/>
+      <c r="BH37" s="10"/>
+      <c r="BI37" s="10"/>
+      <c r="BJ37" s="10"/>
+      <c r="BK37" s="10"/>
+      <c r="BL37" s="10"/>
+      <c r="BM37" s="10"/>
+      <c r="BN37" s="10"/>
+      <c r="BO37" s="10"/>
+      <c r="BP37" s="10"/>
+      <c r="BQ37" s="10"/>
+      <c r="BR37" s="10"/>
+      <c r="BS37" s="10"/>
+      <c r="BT37" s="10"/>
+      <c r="BU37" s="10"/>
+      <c r="BV37" s="10"/>
+      <c r="BW37" s="10"/>
+      <c r="CC37" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="CD37" s="10"/>
+      <c r="CE37" s="10"/>
+      <c r="CF37" s="10"/>
+      <c r="CG37" s="10"/>
+      <c r="CH37" s="10"/>
+      <c r="CI37" s="10"/>
+      <c r="CJ37" s="10"/>
+      <c r="CK37" s="10"/>
+      <c r="CL37" s="10"/>
+      <c r="CM37" s="10"/>
+      <c r="CN37" s="10"/>
+      <c r="CO37" s="10"/>
+      <c r="CP37" s="10"/>
+      <c r="CQ37" s="10"/>
+      <c r="CR37" s="10"/>
+      <c r="CS37" s="10"/>
+      <c r="CT37" s="10"/>
+      <c r="CU37" s="10"/>
+      <c r="CZ37" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="CD37" s="12"/>
-      <c r="CE37" s="12"/>
-      <c r="CF37" s="12"/>
-      <c r="CG37" s="12"/>
-      <c r="CH37" s="12"/>
-      <c r="CI37" s="12"/>
-      <c r="CJ37" s="12"/>
-      <c r="CK37" s="12"/>
-      <c r="CL37" s="12"/>
-      <c r="CM37" s="12"/>
-      <c r="CN37" s="12"/>
-      <c r="CO37" s="12"/>
-      <c r="CP37" s="12"/>
-      <c r="CQ37" s="12"/>
-      <c r="CR37" s="12"/>
-      <c r="CS37" s="12"/>
-      <c r="CT37" s="12"/>
-      <c r="CU37" s="12"/>
-      <c r="CZ37" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="DA37" s="12"/>
-      <c r="DB37" s="12"/>
-      <c r="DC37" s="12"/>
-      <c r="DD37" s="12"/>
-      <c r="DE37" s="12"/>
-      <c r="DF37" s="12"/>
-      <c r="DG37" s="12"/>
-      <c r="DH37" s="12"/>
-      <c r="DI37" s="12"/>
-      <c r="DJ37" s="12"/>
-      <c r="DK37" s="12"/>
-      <c r="DL37" s="12"/>
-      <c r="DM37" s="12"/>
-      <c r="DN37" s="12"/>
-      <c r="DO37" s="12"/>
-      <c r="DP37" s="12"/>
-      <c r="DQ37" s="12"/>
-      <c r="DR37" s="12"/>
+      <c r="DA37" s="10"/>
+      <c r="DB37" s="10"/>
+      <c r="DC37" s="10"/>
+      <c r="DD37" s="10"/>
+      <c r="DE37" s="10"/>
+      <c r="DF37" s="10"/>
+      <c r="DG37" s="10"/>
+      <c r="DH37" s="10"/>
+      <c r="DI37" s="10"/>
+      <c r="DJ37" s="10"/>
+      <c r="DK37" s="10"/>
+      <c r="DL37" s="10"/>
+      <c r="DM37" s="10"/>
+      <c r="DN37" s="10"/>
+      <c r="DO37" s="10"/>
+      <c r="DP37" s="10"/>
+      <c r="DQ37" s="10"/>
+      <c r="DR37" s="10"/>
     </row>
-    <row r="38" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B38" s="6">
-        <v>0</v>
-      </c>
-      <c r="C38" s="6">
-        <v>0</v>
-      </c>
-      <c r="D38" s="6">
-        <v>0</v>
-      </c>
-      <c r="E38" s="6">
+      <c r="B38" s="12">
+        <v>0</v>
+      </c>
+      <c r="C38" s="12">
+        <v>0</v>
+      </c>
+      <c r="D38" s="12">
+        <v>0</v>
+      </c>
+      <c r="E38" s="12">
         <v>4.8328734732758001</v>
       </c>
-      <c r="F38" s="6">
-        <v>0</v>
-      </c>
-      <c r="G38" s="6">
-        <v>0</v>
-      </c>
-      <c r="BE38" s="13" t="s">
+      <c r="F38" s="12">
+        <v>0</v>
+      </c>
+      <c r="G38" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE38" t="s">
+        <v>94</v>
+      </c>
+      <c r="BE38" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="BF38" s="13"/>
-      <c r="BG38" s="13"/>
-      <c r="BH38" s="13"/>
-      <c r="BI38" s="13"/>
-      <c r="BJ38" s="13"/>
-      <c r="BK38" s="13"/>
-      <c r="BL38" s="13"/>
-      <c r="BM38" s="13"/>
-      <c r="BN38" s="13"/>
-      <c r="BO38" s="13"/>
-      <c r="BP38" s="13"/>
-      <c r="BQ38" s="13"/>
-      <c r="BR38" s="13"/>
-      <c r="BS38" s="13"/>
-      <c r="BT38" s="13"/>
-      <c r="BU38" s="13"/>
-      <c r="BV38" s="13"/>
-      <c r="BW38" s="13"/>
+      <c r="BF38" s="11"/>
+      <c r="BG38" s="11"/>
+      <c r="BH38" s="11"/>
+      <c r="BI38" s="11"/>
+      <c r="BJ38" s="11"/>
+      <c r="BK38" s="11"/>
+      <c r="BL38" s="11"/>
+      <c r="BM38" s="11"/>
+      <c r="BN38" s="11"/>
+      <c r="BO38" s="11"/>
+      <c r="BP38" s="11"/>
+      <c r="BQ38" s="11"/>
+      <c r="BR38" s="11"/>
+      <c r="BS38" s="11"/>
+      <c r="BT38" s="11"/>
+      <c r="BU38" s="11"/>
+      <c r="BV38" s="11"/>
+      <c r="BW38" s="11"/>
       <c r="CC38" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B39" s="6">
-        <v>0</v>
-      </c>
-      <c r="C39" s="6">
-        <v>0</v>
-      </c>
-      <c r="D39" s="6">
-        <v>0</v>
-      </c>
-      <c r="E39" s="6">
+      <c r="B39" s="12">
+        <v>0</v>
+      </c>
+      <c r="C39" s="12">
+        <v>0</v>
+      </c>
+      <c r="D39" s="12">
+        <v>0</v>
+      </c>
+      <c r="E39" s="12">
         <v>2.4537243968652998E-2</v>
       </c>
-      <c r="F39" s="6">
-        <v>0</v>
-      </c>
-      <c r="G39" s="6">
+      <c r="F39" s="12">
+        <v>0</v>
+      </c>
+      <c r="G39" s="12">
         <v>0</v>
       </c>
       <c r="BE39" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="40" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B40" s="6">
-        <v>0</v>
-      </c>
-      <c r="C40" s="6">
-        <v>0</v>
-      </c>
-      <c r="D40" s="6">
-        <v>0</v>
-      </c>
-      <c r="E40" s="6">
+      <c r="B40" s="12">
+        <v>0</v>
+      </c>
+      <c r="C40" s="12">
+        <v>0</v>
+      </c>
+      <c r="D40" s="12">
+        <v>0</v>
+      </c>
+      <c r="E40" s="12">
         <v>66.682419111564002</v>
       </c>
-      <c r="F40" s="6">
-        <v>0</v>
-      </c>
-      <c r="G40" s="6">
+      <c r="F40" s="12">
+        <v>0</v>
+      </c>
+      <c r="G40" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B41" s="6">
-        <v>0</v>
-      </c>
-      <c r="C41" s="6">
-        <v>0</v>
-      </c>
-      <c r="D41" s="6">
-        <v>0</v>
-      </c>
-      <c r="E41" s="6">
+      <c r="B41" s="12">
+        <v>0</v>
+      </c>
+      <c r="C41" s="12">
+        <v>0</v>
+      </c>
+      <c r="D41" s="12">
+        <v>0</v>
+      </c>
+      <c r="E41" s="12">
         <v>20.72619293088</v>
       </c>
-      <c r="F41" s="6">
-        <v>0</v>
-      </c>
-      <c r="G41" s="6">
+      <c r="F41" s="12">
+        <v>0</v>
+      </c>
+      <c r="G41" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B42" s="6">
-        <v>0</v>
-      </c>
-      <c r="C42" s="6">
-        <v>0</v>
-      </c>
-      <c r="D42" s="6">
-        <v>0</v>
-      </c>
-      <c r="E42" s="6">
+      <c r="B42" s="12">
+        <v>0</v>
+      </c>
+      <c r="C42" s="12">
+        <v>0</v>
+      </c>
+      <c r="D42" s="12">
+        <v>0</v>
+      </c>
+      <c r="E42" s="12">
         <v>11.722790773811001</v>
       </c>
-      <c r="F42" s="6">
-        <v>0</v>
-      </c>
-      <c r="G42" s="6">
+      <c r="F42" s="12">
+        <v>0</v>
+      </c>
+      <c r="G42" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="6">
-        <v>0</v>
-      </c>
-      <c r="C43" s="6">
-        <v>0</v>
-      </c>
-      <c r="D43" s="6">
-        <v>0</v>
-      </c>
-      <c r="E43" s="6">
+      <c r="B43" s="12">
+        <v>0</v>
+      </c>
+      <c r="C43" s="12">
+        <v>0</v>
+      </c>
+      <c r="D43" s="12">
+        <v>0</v>
+      </c>
+      <c r="E43" s="12">
         <v>351.12025842441</v>
       </c>
-      <c r="F43" s="6">
-        <v>0</v>
-      </c>
-      <c r="G43" s="6">
+      <c r="F43" s="12">
+        <v>0</v>
+      </c>
+      <c r="G43" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B44" s="6">
-        <v>0</v>
-      </c>
-      <c r="C44" s="6">
-        <v>0</v>
-      </c>
-      <c r="D44" s="6">
-        <v>0</v>
-      </c>
-      <c r="E44" s="6">
+      <c r="B44" s="12">
+        <v>0</v>
+      </c>
+      <c r="C44" s="12">
+        <v>0</v>
+      </c>
+      <c r="D44" s="12">
+        <v>0</v>
+      </c>
+      <c r="E44" s="12">
         <v>10.981003594759001</v>
       </c>
-      <c r="F44" s="6">
-        <v>0</v>
-      </c>
-      <c r="G44" s="6">
+      <c r="F44" s="12">
+        <v>0</v>
+      </c>
+      <c r="G44" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B45" s="6">
-        <v>0</v>
-      </c>
-      <c r="C45" s="6">
-        <v>0</v>
-      </c>
-      <c r="D45" s="6">
-        <v>0</v>
-      </c>
-      <c r="E45" s="6">
+      <c r="B45" s="12">
+        <v>0</v>
+      </c>
+      <c r="C45" s="12">
+        <v>0</v>
+      </c>
+      <c r="D45" s="12">
+        <v>0</v>
+      </c>
+      <c r="E45" s="12">
         <v>4.7239291045123002</v>
       </c>
-      <c r="F45" s="6">
-        <v>0</v>
-      </c>
-      <c r="G45" s="6">
+      <c r="F45" s="12">
+        <v>0</v>
+      </c>
+      <c r="G45" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B46" s="6">
+      <c r="B46" s="12">
         <v>148.74389978771001</v>
       </c>
-      <c r="C46" s="6">
-        <v>0</v>
-      </c>
-      <c r="D46" s="6">
-        <v>0</v>
-      </c>
-      <c r="E46" s="6">
-        <v>0</v>
-      </c>
-      <c r="F46" s="6">
-        <v>0</v>
-      </c>
-      <c r="G46" s="6">
+      <c r="C46" s="12">
+        <v>0</v>
+      </c>
+      <c r="D46" s="12">
+        <v>0</v>
+      </c>
+      <c r="E46" s="12">
+        <v>0</v>
+      </c>
+      <c r="F46" s="12">
+        <v>0</v>
+      </c>
+      <c r="G46" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B47" s="6">
-        <v>0</v>
-      </c>
-      <c r="C47" s="6">
-        <v>0</v>
-      </c>
-      <c r="D47" s="6">
-        <v>0</v>
-      </c>
-      <c r="E47" s="6">
+      <c r="B47" s="12">
+        <v>0</v>
+      </c>
+      <c r="C47" s="12">
+        <v>0</v>
+      </c>
+      <c r="D47" s="12">
+        <v>0</v>
+      </c>
+      <c r="E47" s="12">
         <v>1855.3143386280001</v>
       </c>
-      <c r="F47" s="6">
-        <v>0</v>
-      </c>
-      <c r="G47" s="6">
+      <c r="F47" s="12">
+        <v>0</v>
+      </c>
+      <c r="G47" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:122" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:124" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B48" s="6">
-        <v>0</v>
-      </c>
-      <c r="C48" s="6">
-        <v>0</v>
-      </c>
-      <c r="D48" s="6">
-        <v>0</v>
-      </c>
-      <c r="E48" s="6">
+      <c r="B48" s="12">
+        <v>0</v>
+      </c>
+      <c r="C48" s="12">
+        <v>0</v>
+      </c>
+      <c r="D48" s="12">
+        <v>0</v>
+      </c>
+      <c r="E48" s="12">
         <v>73.809561478158003</v>
       </c>
-      <c r="F48" s="6">
-        <v>0</v>
-      </c>
-      <c r="G48" s="6">
+      <c r="F48" s="12">
+        <v>0</v>
+      </c>
+      <c r="G48" s="12">
         <v>0</v>
       </c>
     </row>
@@ -6219,22 +6368,22 @@
       <c r="A49" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B49" s="6">
-        <v>0</v>
-      </c>
-      <c r="C49" s="6">
-        <v>0</v>
-      </c>
-      <c r="D49" s="6">
-        <v>0</v>
-      </c>
-      <c r="E49" s="6">
-        <v>0</v>
-      </c>
-      <c r="F49" s="6">
+      <c r="B49" s="12">
+        <v>0</v>
+      </c>
+      <c r="C49" s="12">
+        <v>0</v>
+      </c>
+      <c r="D49" s="12">
+        <v>0</v>
+      </c>
+      <c r="E49" s="12">
+        <v>0</v>
+      </c>
+      <c r="F49" s="12">
         <v>171.94047456000001</v>
       </c>
-      <c r="G49" s="6">
+      <c r="G49" s="12">
         <v>0</v>
       </c>
     </row>
@@ -6242,44 +6391,44 @@
       <c r="A50" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B50" s="6">
-        <v>0</v>
-      </c>
-      <c r="C50" s="6">
-        <v>0</v>
-      </c>
-      <c r="D50" s="6">
-        <v>0</v>
-      </c>
-      <c r="E50" s="6">
+      <c r="B50" s="12">
+        <v>0</v>
+      </c>
+      <c r="C50" s="12">
+        <v>0</v>
+      </c>
+      <c r="D50" s="12">
+        <v>0</v>
+      </c>
+      <c r="E50" s="12">
         <v>2.1592437759009999</v>
       </c>
-      <c r="F50" s="6">
-        <v>0</v>
-      </c>
-      <c r="G50" s="6">
+      <c r="F50" s="12">
+        <v>0</v>
+      </c>
+      <c r="G50" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C51" s="12"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
-      <c r="G51" s="12"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11"/>
     </row>
     <row r="71" spans="1:52" ht="244" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
@@ -8854,27 +9003,27 @@
       <c r="B91" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K91" s="12" t="s">
+      <c r="K91" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="L91" s="12"/>
-      <c r="M91" s="12"/>
-      <c r="N91" s="12"/>
-      <c r="O91" s="12"/>
-      <c r="P91" s="12"/>
-      <c r="Q91" s="12"/>
-      <c r="R91" s="12"/>
-      <c r="S91" s="12"/>
-      <c r="T91" s="12"/>
-      <c r="U91" s="12"/>
-      <c r="V91" s="12"/>
-      <c r="W91" s="12"/>
-      <c r="X91" s="12"/>
-      <c r="Y91" s="12"/>
-      <c r="Z91" s="12"/>
-      <c r="AA91" s="12"/>
-      <c r="AB91" s="12"/>
-      <c r="AC91" s="12"/>
+      <c r="L91" s="10"/>
+      <c r="M91" s="10"/>
+      <c r="N91" s="10"/>
+      <c r="O91" s="10"/>
+      <c r="P91" s="10"/>
+      <c r="Q91" s="10"/>
+      <c r="R91" s="10"/>
+      <c r="S91" s="10"/>
+      <c r="T91" s="10"/>
+      <c r="U91" s="10"/>
+      <c r="V91" s="10"/>
+      <c r="W91" s="10"/>
+      <c r="X91" s="10"/>
+      <c r="Y91" s="10"/>
+      <c r="Z91" s="10"/>
+      <c r="AA91" s="10"/>
+      <c r="AB91" s="10"/>
+      <c r="AC91" s="10"/>
       <c r="AG91" s="2" t="s">
         <v>78</v>
       </c>
@@ -8940,53 +9089,58 @@
       <c r="B92" t="s">
         <v>79</v>
       </c>
-      <c r="AH92" s="12" t="s">
+      <c r="AH92" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="AI92" s="12"/>
-      <c r="AJ92" s="12"/>
-      <c r="AK92" s="12"/>
-      <c r="AL92" s="12"/>
-      <c r="AM92" s="12"/>
-      <c r="AN92" s="12"/>
-      <c r="AO92" s="12"/>
-      <c r="AP92" s="12"/>
-      <c r="AQ92" s="12"/>
-      <c r="AR92" s="12"/>
-      <c r="AS92" s="12"/>
-      <c r="AT92" s="12"/>
-      <c r="AU92" s="12"/>
-      <c r="AV92" s="12"/>
-      <c r="AW92" s="12"/>
-      <c r="AX92" s="12"/>
-      <c r="AY92" s="12"/>
-      <c r="AZ92" s="12"/>
+      <c r="AI92" s="10"/>
+      <c r="AJ92" s="10"/>
+      <c r="AK92" s="10"/>
+      <c r="AL92" s="10"/>
+      <c r="AM92" s="10"/>
+      <c r="AN92" s="10"/>
+      <c r="AO92" s="10"/>
+      <c r="AP92" s="10"/>
+      <c r="AQ92" s="10"/>
+      <c r="AR92" s="10"/>
+      <c r="AS92" s="10"/>
+      <c r="AT92" s="10"/>
+      <c r="AU92" s="10"/>
+      <c r="AV92" s="10"/>
+      <c r="AW92" s="10"/>
+      <c r="AX92" s="10"/>
+      <c r="AY92" s="10"/>
+      <c r="AZ92" s="10"/>
     </row>
     <row r="93" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="AH93" s="13" t="s">
+      <c r="AH93" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="AI93" s="13"/>
-      <c r="AJ93" s="13"/>
-      <c r="AK93" s="13"/>
-      <c r="AL93" s="13"/>
-      <c r="AM93" s="13"/>
-      <c r="AN93" s="13"/>
-      <c r="AO93" s="13"/>
-      <c r="AP93" s="13"/>
-      <c r="AQ93" s="13"/>
-      <c r="AR93" s="13"/>
-      <c r="AS93" s="13"/>
-      <c r="AT93" s="13"/>
-      <c r="AU93" s="13"/>
-      <c r="AV93" s="13"/>
-      <c r="AW93" s="13"/>
-      <c r="AX93" s="13"/>
-      <c r="AY93" s="13"/>
-      <c r="AZ93" s="13"/>
+      <c r="AI93" s="11"/>
+      <c r="AJ93" s="11"/>
+      <c r="AK93" s="11"/>
+      <c r="AL93" s="11"/>
+      <c r="AM93" s="11"/>
+      <c r="AN93" s="11"/>
+      <c r="AO93" s="11"/>
+      <c r="AP93" s="11"/>
+      <c r="AQ93" s="11"/>
+      <c r="AR93" s="11"/>
+      <c r="AS93" s="11"/>
+      <c r="AT93" s="11"/>
+      <c r="AU93" s="11"/>
+      <c r="AV93" s="11"/>
+      <c r="AW93" s="11"/>
+      <c r="AX93" s="11"/>
+      <c r="AY93" s="11"/>
+      <c r="AZ93" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="CC37:CU37"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="CZ37:DR37"/>
+    <mergeCell ref="K91:AC91"/>
+    <mergeCell ref="AH92:AZ92"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="K9:P9"/>
     <mergeCell ref="AH9:AM9"/>
@@ -8997,13 +9151,9 @@
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="K37:AD37"/>
     <mergeCell ref="AH37:BA37"/>
-    <mergeCell ref="CC37:CU37"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="CZ37:DR37"/>
-    <mergeCell ref="K91:AC91"/>
-    <mergeCell ref="AH92:AZ92"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>